<commit_message>
buda publish excel updated
</commit_message>
<xml_diff>
--- a/buda/data/mp4_publish_tracker.xlsx
+++ b/buda/data/mp4_publish_tracker.xlsx
@@ -3613,7 +3613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E189"/>
+  <dimension ref="A1:E255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>“無欲則剛”四字含義，其實修行人都解讀錯了，高僧開示是這種境界！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>“善”和“惡”字拆開看，才明白《法句經》，早已教導如何行善積德！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2025-07-03 04:59:14</t>
+          <t>2025-08-28 04:59:14</t>
         </is>
       </c>
     </row>
@@ -3720,7 +3720,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>”觀自在“三字的含義，其實眾生都理解錯了，原來是這般的境界！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>“妄念”竟是開悟鑰匙？達摩祖師傳下“轉念秘法”，比坐禪十年更有效!#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -3731,7 +3731,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2025-07-03 16:59:14</t>
+          <t>2025-08-29 04:59:14</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>《六祖壇經》裏泄露天機的五句話：修行有成，「三身」便是成果。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>“恩”和“怨”字拆開看，才明白《華嚴經》，早已講明人生一場修行！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -3754,7 +3754,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2025-06-04 04:55:22</t>
+          <t>2025-08-30 04:59:14</t>
         </is>
       </c>
     </row>
@@ -3766,7 +3766,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>《心經》結尾咒語：“揭諦揭諦”是什麼意思？99%的人都理解錯了！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>“明心見性”四字的本意，修行人大多解讀錯誤，六祖揭示是這樣的境界！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -3777,7 +3777,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2025-06-04 10:55:22</t>
+          <t>2025-08-31 04:59:14</t>
         </is>
       </c>
     </row>
@@ -3789,7 +3789,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>《心經》隱藏的秘密，何為”諸法空相“，它不是虛無而是無限可能。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>“無欲則剛”四字含義，其實修行人都解讀錯了，高僧開示是這種境界！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -3800,7 +3800,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2025-06-04 16:55:22</t>
+          <t>2025-07-03 04:59:14</t>
         </is>
       </c>
     </row>
@@ -3812,7 +3812,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>《成唯識論》揭示，末法時代聖者現世五大征兆，輪回五層次的奧秘。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>“看破紅塵”四個字的含義，大部分修行人都理解錯了，高僧開示是這種境界#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -3823,7 +3823,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2025-06-04 22:55:22</t>
+          <t>2025-09-01 04:59:14</t>
         </is>
       </c>
     </row>
@@ -3835,7 +3835,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>《楞嚴經》到底是真經還是偽經？佛教界與學術界最大的爭論。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>“眾生平等”四字的含義，其實學佛人都理解錯了，佛陀開示是這種境界！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2025-07-04 04:59:14</t>
+          <t>2025-09-02 04:59:14</t>
         </is>
       </c>
     </row>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>《金剛經》中隱藏的神秘智慧，竟是消除一切煩惱的法門。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>“色即是空”四字的真相，大眾普遍理解有偏差，高僧開示正確的含義#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2025-07-04 16:59:14</t>
+          <t>2025-09-03 04:59:14</t>
         </is>
       </c>
     </row>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>《金剛經》精髓：見性成佛不在文字，而在參透九字真言！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>“菩提心”三個字，決定了你修行的成敗，很多人都誤解了它的真意！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -3892,7 +3892,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2025-07-05 04:59:14</t>
+          <t>2025-09-04 04:59:14</t>
         </is>
       </c>
     </row>
@@ -3904,7 +3904,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>「三世佛」都是誰？佛教時間與空間哲學的終極解讀。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>”觀自在“三字的含義，其實眾生都理解錯了，原來是這般的境界！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2025-07-05 16:59:14</t>
+          <t>2025-07-03 16:59:14</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>一個視頻講透《心經》核心理論「緣起性空」，擺脫煩惱的終極智慧。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>《六祖壇經》裏泄露天機的五句話：修行有成，「三身」便是成果。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -3938,7 +3938,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2025-07-06 04:59:14</t>
+          <t>2025-06-04 04:55:22</t>
         </is>
       </c>
     </row>
@@ -3950,7 +3950,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>不去掃墓就是不孝嗎？廣欽老和尚的開示，讓人明白了真正的孝道。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>《心經》260個字藏著什麼天機？玄奘法師說讀懂這一句，就能看破生死輪迴。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -3961,7 +3961,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2025-06-05 22:55:22</t>
+          <t>2025-09-05 04:59:14</t>
         </is>
       </c>
     </row>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>不知乞討的人真假，到底要不要布施，高僧一句話點醒迷茫！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>《心經》結尾咒語：“揭諦揭諦”是什麼意思？99%的人都理解錯了！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2025-06-05 04:55:22</t>
+          <t>2025-06-04 10:55:22</t>
         </is>
       </c>
     </row>
@@ -3996,7 +3996,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>不要懼怕任何人和事，佛陀傳授五觀察法，面對一切險境可心如止水！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>《心經》隱藏的秘密，何為”諸法空相“，它不是虛無而是無限可能。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -4007,7 +4007,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2025-07-06 16:59:14</t>
+          <t>2025-06-04 16:55:22</t>
         </is>
       </c>
     </row>
@@ -4019,7 +4019,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>二十分鐘講透佛教的三界與六道，釋迦牟尼不為人知的宇宙！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>《成唯識論》揭示，末法時代聖者現世五大征兆，輪回五層次的奧秘。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -4030,7 +4030,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2025-06-05 10:55:22</t>
+          <t>2025-06-04 22:55:22</t>
         </is>
       </c>
     </row>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>什麽是「三皈五戒」？真正能改變人生軌跡的佛教智慧。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>《楞嚴經》到底是真經還是偽經？佛教界與學術界最大的爭論。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -4053,7 +4053,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2025-07-07 04:59:14</t>
+          <t>2025-07-04 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4065,7 +4065,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>佛學中的「禪」有何意義？修行者「覺悟」的終極智慧。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>《法華經》七萬字中，這五句話藏著三界六道輪迴的終極真相，破迷開悟!#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -4076,7 +4076,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2025-06-05 16:55:22</t>
+          <t>2025-09-06 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4088,7 +4088,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>佛教七大密咒，竟隱藏能量共振原理，持念消災增福奧祕解析。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>《無量壽經》六重妙義，第三重最圓融玄妙，悟者得度但鳳毛麟角#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -4099,7 +4099,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2025-06-06 04:55:22</t>
+          <t>2025-09-07 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>佛教千年難解的謎題，業報到底是誰的？前世所做你該承擔嗎？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>《金剛經》中隱藏的神秘智慧，竟是消除一切煩惱的法門。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2025-07-07 16:59:14</t>
+          <t>2025-07-04 16:59:14</t>
         </is>
       </c>
     </row>
@@ -4134,7 +4134,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>佛教所說的極樂世界到底在哪裏？念佛真的能脫離輪回嗎？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>《金剛經》精髓：見性成佛不在文字，而在參透九字真言！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -4145,7 +4145,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2025-06-09 04:59:14</t>
+          <t>2025-07-05 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4157,7 +4157,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>佛教的三千大千世界究竟有多大？他與科學的宇宙觀有什麽共通點？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>「三世佛」都是誰？佛教時間與空間哲學的終極解讀。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -4168,7 +4168,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2025-06-09 10:59:14</t>
+          <t>2025-07-05 16:59:14</t>
         </is>
       </c>
     </row>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>佛教的四大菩薩都是誰？他們如何成就眾生的覺悟之路。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>一個視頻講透《心經》核心理論「緣起性空」，擺脫煩惱的終極智慧。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2025-06-09 16:59:14</t>
+          <t>2025-07-06 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4203,7 +4203,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>佛教的最高真理，中道智慧，超越對立終極覺悟的奧祕！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>不去掃墓就是不孝嗎？廣欽老和尚的開示，讓人明白了真正的孝道。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2025-06-09 22:59:14</t>
+          <t>2025-06-05 22:55:22</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>佛法三境界，空為無執、色為顯相、幻為虛妄，參透關鍵即得大解脫。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>不知乞討的人真假，到底要不要布施，高僧一句話點醒迷茫！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -4237,7 +4237,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2025-06-10 04:59:14</t>
+          <t>2025-06-05 04:55:22</t>
         </is>
       </c>
     </row>
@@ -4249,7 +4249,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>佛法如何顛覆現代焦慮，99%的人從未嘗試過的生活禪修之道！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>不要因小事而焦慮，佛陀教誨“忍辱”功德，化解怨恨成就內心強大#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -4260,7 +4260,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2025-07-08 04:59:14</t>
+          <t>2025-09-08 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>佛法的悖論，為何“無我”還要“輪迴”，到底是誰在承受因果？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>不要執著完美人設，佛陀開示中道智慧，擁抱不完美才能活出真我#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2025-06-10 10:59:14</t>
+          <t>2025-09-09 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4295,7 +4295,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>佛道雙修！超越凡俗的修行秘訣，從煉氣入門到陽神出遊的完整指引！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>不要害怕衰老病痛，佛陀傳授慈心觀修持法，讓身心在困境中安寧自在！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4306,7 +4306,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2025-06-10 16:59:14</t>
+          <t>2025-09-10 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4318,7 +4318,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>佛門內部千年爭議，高僧大德為何質疑輪迴？玄奘法師的解答令人深思！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>不要懷疑任何佛與法，佛陀宣講三皈依，堅定信仰可獲得加持！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4329,7 +4329,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2025-07-08 16:59:14</t>
+          <t>2025-09-11 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>佛門謎題，究竟在七大佛祖中，誰才是真正的萬佛之祖？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>不要懼怕任何人和事，佛陀傳授五觀察法，面對一切險境可心如止水！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4352,7 +4352,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2025-07-09 04:59:14</t>
+          <t>2025-07-06 16:59:14</t>
         </is>
       </c>
     </row>
@@ -4364,7 +4364,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>佛陀2500年前已發現，宇宙最神祕力量，因果相續如何影響命運。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>二十分鐘講透佛教的三界與六道，釋迦牟尼不為人知的宇宙！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4375,7 +4375,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2025-06-10 22:59:14</t>
+          <t>2025-06-05 10:55:22</t>
         </is>
       </c>
     </row>
@@ -4387,7 +4387,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>佛陀2500年前的預言，五濁惡世已降臨，解脫之道就在這裏。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>五台山供米爭議越鬧越大：佛陀早在千年涅槃前，就開示供養布施真諦！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2025-06-11 04:59:14</t>
+          <t>2025-09-12 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4410,7 +4410,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>佛陀三身之謎，法身、報身、應身，哪一身才是真正的佛？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>什麽是「三皈五戒」？真正能改變人生軌跡的佛教智慧。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4421,7 +4421,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2025-06-11 10:59:14</t>
+          <t>2025-07-07 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4433,7 +4433,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>佛陀在燈下為弟子講解，影子消失的道理，原來這才是真正的解脫！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛學中的「禪」有何意義？修行者「覺悟」的終極智慧。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4444,7 +4444,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2025-06-11 16:59:14</t>
+          <t>2025-06-05 16:55:22</t>
         </is>
       </c>
     </row>
@@ -4456,7 +4456,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>佛陀慈悲開示，信佛要必知這三句話，修行之路自然順暢無礙！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛教七大密咒，竟隱藏能量共振原理，持念消災增福奧祕解析。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2025-07-09 16:59:14</t>
+          <t>2025-06-06 04:55:22</t>
         </is>
       </c>
     </row>
@@ -4479,7 +4479,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>佛陀慈悲開示，這七種無財布施法，不用花錢也能獲大福報。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛教千年難解的謎題，業報到底是誰的？前世所做你該承擔嗎？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4490,7 +4490,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2025-06-11 22:59:14</t>
+          <t>2025-07-07 16:59:14</t>
         </is>
       </c>
     </row>
@@ -4502,7 +4502,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>佛陀慈悲開示：五蘊皆空之後還有一物，悟此可直接超越三界。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛教所說的極樂世界到底在哪裏？念佛真的能脫離輪回嗎？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -4513,7 +4513,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2025-06-12 04:59:14</t>
+          <t>2025-06-09 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4525,7 +4525,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>佛陀慈悲開示：每個人身上的疾病，其實是前世所欠之債的清算。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛教的“不執著”與道家的“無為而治”有何聯繫？竟指向著同一個真理？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -4534,7 +4534,11 @@
       <c r="D40" t="n">
         <v>1</v>
       </c>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2025-09-13 04:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4544,7 +4548,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>佛陀涅槃前點化迦葉，真修行者不拘泥形式，而是通達這四種內心境界。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛教的三千大千世界究竟有多大？他與科學的宇宙觀有什麽共通點？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -4553,7 +4557,11 @@
       <c r="D41" t="n">
         <v>1</v>
       </c>
-      <c r="E41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2025-06-09 10:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4563,7 +4571,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>佛陀用一片落葉，向阿難開示驚人秘密，我不是第一位佛。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛教的四大菩薩都是誰？他們如何成就眾生的覺悟之路。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -4572,7 +4580,11 @@
       <c r="D42" t="n">
         <v>1</v>
       </c>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2025-06-09 16:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4582,7 +4594,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>佛陀的五時說法到底是什麽？從華嚴到涅槃，成佛的秘密就在這裏！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛教的最高真理，中道智慧，超越對立終極覺悟的奧祕！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -4593,7 +4605,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2025-06-12 10:59:14</t>
+          <t>2025-06-09 22:59:14</t>
         </is>
       </c>
     </row>
@@ -4605,7 +4617,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>佛陀的女弟子蓮華色，曾犯下亂倫罪過的她，是如何修成神通第一的。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛法三境界，空為無執、色為顯相、幻為虛妄，參透關鍵即得大解脫。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -4616,7 +4628,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2025-06-12 16:59:14</t>
+          <t>2025-06-10 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4628,7 +4640,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>佛陀的矛盾指引，放下慾望卻要成佛，揭秘背後的驚人智慧！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛法如何顛覆現代焦慮，99%的人從未嘗試過的生活禪修之道！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -4639,7 +4651,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2025-06-12 22:59:14</t>
+          <t>2025-07-08 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4663,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>佛陀祕傳居家八法，在家修行人虔心領悟，今生來世皆安樂。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛法智慧：人過五十，切記守住這“三樣東西”，晚年才能安穩幸福！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -4660,7 +4672,11 @@
       <c r="D46" t="n">
         <v>1</v>
       </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2025-09-14 04:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4670,7 +4686,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>佛陀說眾生皆可成佛，為何我們還在輪回？原來缺失最重要的三步。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛法的悖論，為何“無我”還要“輪迴”，到底是誰在承受因果？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -4681,7 +4697,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2025-06-13 04:59:14</t>
+          <t>2025-06-10 10:59:14</t>
         </is>
       </c>
     </row>
@@ -4693,7 +4709,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>佛陀開示弟子：夫妻緣分從何而來，今生相遇有何因果聯繫？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛道雙修！超越凡俗的修行秘訣，從煉氣入門到陽神出遊的完整指引！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -4704,7 +4720,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2025-06-13 10:59:14</t>
+          <t>2025-06-10 16:59:14</t>
         </is>
       </c>
     </row>
@@ -4716,7 +4732,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>佛陀開示眾弟子：命中注定與自由意志，到底該如何平衡！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛門內部千年爭議，高僧大德為何質疑輪迴？玄奘法師的解答令人深思！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -4727,7 +4743,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2025-06-13 16:59:14</t>
+          <t>2025-07-08 16:59:14</t>
         </is>
       </c>
     </row>
@@ -4739,7 +4755,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>佛陀開示阿難：心不在身內，也不在身外！阿難聽後頓時茅塞頓開。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛門謎題，究竟在七大佛祖中，誰才是真正的萬佛之祖？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -4748,7 +4764,11 @@
       <c r="D50" t="n">
         <v>1</v>
       </c>
-      <c r="E50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2025-07-09 04:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4758,7 +4778,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>佛陀開示：命中有時終須有，人生這3件事早有安排，順勢而為！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀2500年前已發現，宇宙最神祕力量，因果相續如何影響命運。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -4769,7 +4789,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2025-06-13 22:59:14</t>
+          <t>2025-06-10 22:59:14</t>
         </is>
       </c>
     </row>
@@ -4781,7 +4801,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>佛陀點化阿難，真假佛法怎麽分辨，真正佛法的四大標誌。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀2500年前的預言，五濁惡世已降臨，解脫之道就在這裏。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -4792,7 +4812,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2025-06-14 04:59:14</t>
+          <t>2025-06-11 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4804,7 +4824,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>佛陀點化阿難：修行人每天進行五種觀想，才能真正自在解脫！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀一句反問，讓須菩提當場開悟！破解“五蘊皆空”真諦！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -4815,7 +4835,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2025-07-10 04:59:14</t>
+          <t>2025-09-15 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4827,7 +4847,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>佛陀點破夫妻因果：為何夫妻緣盡便成冤？三世因果早已註定。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀三身之謎，法身、報身、應身，哪一身才是真正的佛？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -4838,7 +4858,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2025-06-14 10:59:14</t>
+          <t>2025-06-11 10:59:14</t>
         </is>
       </c>
     </row>
@@ -4850,7 +4870,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>你對誰生嗔恨，就會與誰轉世為親，因果業力循環藏何秘密？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀在燈下為弟子講解，影子消失的道理，原來這才是真正的解脫！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -4859,7 +4879,11 @@
       <c r="D55" t="n">
         <v>1</v>
       </c>
-      <c r="E55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2025-06-11 16:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4869,7 +4893,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>修行者到底能不能吃雞蛋？印光大師的開示，道出佛教戒律真諦。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀宣講《圓覺經》，“知幻即離”這四個字，揭示了最深奧的修行要訣#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -4880,7 +4904,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>2025-06-14 16:59:14</t>
+          <t>2025-09-16 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4892,7 +4916,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>修行路上的三大障礙：眼淫、心淫、意淫，龍樹菩薩親傳破解奧秘！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀宣講六度波羅蜜：為何布施能獲得財富？六度修行的神奇變化讓人震驚！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -4901,7 +4925,11 @@
       <c r="D57" t="n">
         <v>1</v>
       </c>
-      <c r="E57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2025-09-17 04:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4911,7 +4939,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>全球人口負增長，六道輪迴也會重組嗎？文殊菩薩揭示五大奧祕！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀慈悲開示，信佛要必知這三句話，修行之路自然順暢無礙！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -4922,7 +4950,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2025-06-14 22:59:14</t>
+          <t>2025-07-09 16:59:14</t>
         </is>
       </c>
     </row>
@@ -4934,7 +4962,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>六祖慧能金身千年不腐，卻遭遇3次劫難，最後1次幾乎被毀！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀慈悲開示，這七種無財布施法，不用花錢也能獲大福報。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -4945,7 +4973,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2025-06-15 04:59:14</t>
+          <t>2025-06-11 22:59:14</t>
         </is>
       </c>
     </row>
@@ -4957,7 +4985,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>六祖慧能開示：不要羨慕有才華之人，見性後方知天賦真相！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀慈悲開示：五蘊皆空之後還有一物，悟此可直接超越三界。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -4968,7 +4996,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2025-07-11 04:59:14</t>
+          <t>2025-06-12 04:59:14</t>
         </is>
       </c>
     </row>
@@ -4980,7 +5008,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>六祖慧能點化：做這件事可消三生罪業，福報不請自來。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀慈悲開示：每個人身上的疾病，其實是前世所欠之債的清算。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -4989,11 +5017,7 @@
       <c r="D61" t="n">
         <v>1</v>
       </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>2025-06-15 10:59:14</t>
-        </is>
-      </c>
+      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5003,7 +5027,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>刀師村長質問佛陀，佛法普渡眾生了嗎？佛陀用兩個比喻揭示傳法真諦。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀涅槃前點化迦葉，真修行者不拘泥形式，而是通達這四種內心境界。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -5012,11 +5036,7 @@
       <c r="D62" t="n">
         <v>1</v>
       </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>2025-06-15 16:59:14</t>
-        </is>
-      </c>
+      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5026,7 +5046,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>十四分鐘徹底讀懂《心經》，260字竟隱藏著成佛奧秘。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀用一片落葉，向阿難開示驚人秘密，我不是第一位佛。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -5035,11 +5055,7 @@
       <c r="D63" t="n">
         <v>1</v>
       </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>2025-06-15 22:59:14</t>
-        </is>
-      </c>
+      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5049,7 +5065,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>唵嘛呢叭咪吽有何奧妙？藥師佛揭示：六字真言蘊含的不凡能量。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀的“緣起性空”與老子的“道法自然”有何關係？兩個概念似乎相同#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -5058,7 +5074,11 @@
       <c r="D64" t="n">
         <v>1</v>
       </c>
-      <c r="E64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2025-09-18 04:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5068,7 +5088,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>因果報應有多可怕，佛陀親口警示，修行者絕對不能觸碰的3大禁忌。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀的五時說法到底是什麽？從華嚴到涅槃，成佛的秘密就在這裏！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -5077,7 +5097,11 @@
       <c r="D65" t="n">
         <v>1</v>
       </c>
-      <c r="E65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2025-06-12 10:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5087,7 +5111,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>地藏王菩薩告誡：人去世後到陰間必經這九關，看完生前必修功德。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀的女弟子蓮華色，曾犯下亂倫罪過的她，是如何修成神通第一的。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -5098,7 +5122,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>2025-06-16 04:59:14</t>
+          <t>2025-06-12 16:59:14</t>
         </is>
       </c>
     </row>
@@ -5110,7 +5134,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>地藏王菩薩巡視地獄，發現兩亡魂不願輪回，菩薩的教誨讓人頓悟。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀的矛盾指引，放下慾望卻要成佛，揭秘背後的驚人智慧！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -5121,7 +5145,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2025-07-12 04:59:14</t>
+          <t>2025-06-12 22:59:14</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5157,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>地藏王菩薩揭示，清明節不要隨便燒紙錢，這三樣才是亡者真正需要。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀祕傳居家八法，在家修行人虔心領悟，今生來世皆安樂。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -5142,11 +5166,7 @@
       <c r="D68" t="n">
         <v>1</v>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>2025-06-16 10:59:14</t>
-        </is>
-      </c>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5156,7 +5176,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>地藏王菩薩秘傳：為何通靈之人多磨難？與鬼神往來注意四大禁忌！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀說眾生皆可成佛，為何我們還在輪回？原來缺失最重要的三步。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -5167,7 +5187,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>2025-07-13 04:59:14</t>
+          <t>2025-06-13 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5179,7 +5199,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>地藏王菩薩開示：頭七超度的重要意義，這七天對亡者至關重要。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀開示壽命玄機：人到老年有兩個坎，過則長壽安康！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -5190,7 +5210,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2025-06-16 16:59:14</t>
+          <t>2025-09-19 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5202,7 +5222,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>地藏王菩薩點化：想要來世有善報的人，今生要常做這五件事！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀開示弟子：夫妻緣分從何而來，今生相遇有何因果聯繫？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -5213,7 +5233,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2025-07-14 04:59:14</t>
+          <t>2025-06-13 10:59:14</t>
         </is>
       </c>
     </row>
@@ -5225,7 +5245,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>地藏王菩薩：少跟孩子置氣，他們選擇你為父母，有這三種原因！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀開示眾弟子：命中注定與自由意志，到底該如何平衡！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -5236,7 +5256,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>2025-06-16 22:59:14</t>
+          <t>2025-06-13 16:59:14</t>
         </is>
       </c>
     </row>
@@ -5248,7 +5268,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>外道沙門師傅詆毀佛法，眾比丘憤而議論，佛陀的教誨令所有人頓悟。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀開示阿難三我：本我，自我，真我！一旦看清自我就修行圓滿了。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -5259,7 +5279,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2025-06-17 04:59:14</t>
+          <t>2025-09-20 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5291,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>大勢至菩薩開示：人在投胎前，為何會自己選擇父母，背後原因令人深思。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀開示阿難：心不在身內，也不在身外！阿難聽後頓時茅塞頓開。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -5280,11 +5300,7 @@
       <c r="D74" t="n">
         <v>1</v>
       </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>2025-06-17 10:59:14</t>
-        </is>
-      </c>
+      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5294,7 +5310,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>大勢至菩薩開示：末法時代紛擾世界，保持內心平靜的終極奧秘！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀開示：命中有時終須有，人生這3件事早有安排，順勢而為！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -5305,7 +5321,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>2025-06-17 16:59:14</t>
+          <t>2025-06-13 22:59:14</t>
         </is>
       </c>
     </row>
@@ -5317,7 +5333,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>大勢至菩薩點化：當六根不凈時，這個修行秘訣讓你立刻心如止水。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀點化阿難，真假佛法怎麽分辨，真正佛法的四大標誌。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -5328,7 +5344,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2025-06-17 22:59:14</t>
+          <t>2025-06-14 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5340,7 +5356,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>大梵天王問佛陀：何為空中妙有？佛陀回答揭示覺知奧秘。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀點化阿難：修行人每天進行五種觀想，才能真正自在解脫！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -5351,7 +5367,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>2025-06-18 04:59:14</t>
+          <t>2025-07-10 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5363,7 +5379,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>大迦葉問佛陀，為何修行人要斷除色欲？元神外泄導致修行受阻。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>佛陀點破夫妻因果：為何夫妻緣盡便成冤？三世因果早已註定。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -5372,7 +5388,11 @@
       <c r="D78" t="n">
         <v>1</v>
       </c>
-      <c r="E78" t="inlineStr"/>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>2025-06-14 10:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5382,7 +5402,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>大迦葉問佛陀：為何亡者於人間徘徊七日，佛陀揭示陰陽兩界奧秘。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>你對誰生嗔恨，就會與誰轉世為親，因果業力循環藏何秘密？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -5391,11 +5411,7 @@
       <c r="D79" t="n">
         <v>1</v>
       </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>2025-06-18 10:59:14</t>
-        </is>
-      </c>
+      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5405,7 +5421,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>大迦葉問釋迦牟尼：成佛前為何要履行生子義務？真相讓所有人覺悟！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>修行者到底能不能吃雞蛋？印光大師的開示，道出佛教戒律真諦。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -5416,7 +5432,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2025-06-18 16:59:14</t>
+          <t>2025-06-14 16:59:14</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5444,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>夫妻合葬輪迴後就能相見？地藏王菩薩說：來世能否重逢看這三件事！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>修行路上的三大障礙：眼淫、心淫、意淫，龍樹菩薩親傳破解奧秘！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -5437,11 +5453,7 @@
       <c r="D81" t="n">
         <v>1</v>
       </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>2025-07-15 04:59:14</t>
-        </is>
-      </c>
+      <c r="E81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -5451,7 +5463,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>女子跪問佛陀，為何不能散父親骨灰？佛陀揭示輪回奧秘。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>全球人口負增長，六道輪迴也會重組嗎？文殊菩薩揭示五大奧祕！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -5462,7 +5474,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>2025-06-18 22:59:14</t>
+          <t>2025-06-14 22:59:14</t>
         </is>
       </c>
     </row>
@@ -5474,7 +5486,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>學佛之人切記，千萬別做這三件事，會耗光你的福報。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>六祖慧能圓寂前開示：因果定律無人能改，但有一事例外#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -5485,7 +5497,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>2025-06-19 04:59:14</t>
+          <t>2025-09-21 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5497,7 +5509,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>學佛人不可不知，佛前十種供品的寓意和果報，正確供養才能修行圓滿。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>六祖慧能生前開示：萬法歸一皆是假相，只有這四個修行是真機#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -5508,7 +5520,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2025-06-19 10:59:14</t>
+          <t>2025-09-22 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5520,7 +5532,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>家裡有“髒東西”怎麼辦？持念這一佛教咒語，驅邪避凶最為靈驗！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>六祖慧能臨終警醒世人，修行人大多數都是自欺，見性成佛就在這兩個關鍵!#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -5531,7 +5543,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2025-06-19 16:59:14</t>
+          <t>2025-09-23 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5543,7 +5555,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>富樓那問釋迦牟尼：您說無生無滅，那麽哪來的六道輪回呢？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>六祖慧能說“無輪迴可出”，這句話究竟是什麼意思？一個公案道破玄機#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -5554,7 +5566,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>2025-06-19 22:59:14</t>
+          <t>2025-09-24 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5566,7 +5578,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>已故親人會思念陽間人嗎？地藏王菩薩開示：時常思念但多數人不知！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>六祖慧能金身千年不腐，卻遭遇3次劫難，最後1次幾乎被毀！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -5577,7 +5589,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>2025-07-16 04:59:14</t>
+          <t>2025-06-15 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5589,7 +5601,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>帝釋天三問釋迦牟尼：「何為善」？佛陀的回答揭示人生大智慧。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>六祖慧能開示：不要羨慕有才華之人，見性後方知天賦真相！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -5600,7 +5612,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>2025-06-20 04:59:14</t>
+          <t>2025-07-11 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5612,7 +5624,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>帝釋天三問釋迦牟尼：輪回的盡頭是什麽？佛陀的開示令所有人頓悟！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>六祖慧能開示：禪宗開悟終極心法不在參禪，而在心性本空的循環法則#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -5623,7 +5635,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>2025-06-20 10:59:14</t>
+          <t>2025-09-25 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5635,7 +5647,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>帝釋天問佛陀：何為菩提心？佛陀只用三個字，讓在場修行者瞬間開悟。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>六祖慧能點化：做這件事可消三生罪業，福報不請自來。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -5646,7 +5658,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>2025-06-20 16:59:14</t>
+          <t>2025-06-15 10:59:14</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5670,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>廣欽老和尚開示，如何做到一心不亂，領悟這三點當下即解脫！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>刀師村長質問佛陀，佛法普渡眾生了嗎？佛陀用兩個比喻揭示傳法真諦。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -5669,7 +5681,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>2025-06-20 22:59:14</t>
+          <t>2025-06-15 16:59:14</t>
         </is>
       </c>
     </row>
@@ -5681,7 +5693,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>彌勒佛問佛陀，何為究竟解脫，一句話讓眾人頓悟涅槃。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>十四分鐘徹底讀懂《心經》，260字竟隱藏著成佛奧秘。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -5692,7 +5704,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>2025-06-21 04:59:14</t>
+          <t>2025-06-15 22:59:14</t>
         </is>
       </c>
     </row>
@@ -5704,7 +5716,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>彌勒佛開示：人世間最大的布施，不是錢財而是這四個字！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>印光大師臨終前說：凈土法門有訣竅，八字箴言點透念佛要義!#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -5715,7 +5727,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>2025-07-17 04:59:14</t>
+          <t>2025-09-26 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5727,7 +5739,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>彌勒菩薩指引，轉世的真諦是什麼？超越生死才是究竟解脫！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>唵嘛呢叭咪吽有何奧妙？藥師佛揭示：六字真言蘊含的不凡能量。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -5736,11 +5748,7 @@
       <c r="D94" t="n">
         <v>1</v>
       </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>2025-06-21 10:59:14</t>
-        </is>
-      </c>
+      <c r="E94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5750,7 +5758,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>心經中“究竟涅槃”的境界是什麼？大勢至菩薩的開示，讓眾人悟道修行真諦。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>四大皆空的真正含義：現代修行人都理解錯了，佛陀開示是這般境界！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -5761,7 +5769,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>2025-06-21 16:59:14</t>
+          <t>2025-09-27 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5773,7 +5781,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>念佛不見佛現身，我們到底在求誰，禪師點破道理妙不可言！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>因果報應有多可怕，佛陀親口警示，修行者絕對不能觸碰的3大禁忌。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -5782,11 +5790,7 @@
       <c r="D96" t="n">
         <v>1</v>
       </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>2025-06-21 22:59:14</t>
-        </is>
-      </c>
+      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5796,7 +5800,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>念佛人的死後因果，觀世音菩薩揭秘：念佛次數決定往生品位！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>在家居士能開悟成佛嗎？修行方式與成就高低，佛陀有明確規定！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -5807,7 +5811,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>2025-07-18 04:59:14</t>
+          <t>2025-09-28 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5819,7 +5823,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>意淫比實淫更損元氣，未除此障修行難成就，學會此法可根除！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>地藏王菩薩告誡：人去世後到陰間必經這九關，看完生前必修功德。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -5830,7 +5834,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>2025-07-19 04:59:14</t>
+          <t>2025-06-16 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5842,7 +5846,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>探索密教深奧智慧！揭示寧瑪派傳世秘法與大圓滿修行的真實內涵！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>地藏王菩薩巡視地獄，發現兩亡魂不願輪回，菩薩的教誨讓人頓悟。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -5853,7 +5857,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>2025-06-22 04:59:14</t>
+          <t>2025-07-12 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5865,7 +5869,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>揭開「阿彌陀佛」與「釋迦牟尼佛」的神秘關系，讓你徹底理解佛教宇宙的無盡智慧。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>地藏王菩薩揭示，清明節不要隨便燒紙錢，這三樣才是亡者真正需要。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -5876,7 +5880,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>2025-07-20 04:59:14</t>
+          <t>2025-06-16 10:59:14</t>
         </is>
       </c>
     </row>
@@ -5888,7 +5892,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>文殊菩薩問釋迦牟尼：何為無上正覺？佛陀的回答讓众人醍醐灌頂。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>地藏王菩薩秘傳：為何通靈之人多磨難？與鬼神往來注意四大禁忌！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -5899,7 +5903,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>2025-06-22 10:59:14</t>
+          <t>2025-07-13 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5911,7 +5915,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>文殊菩薩開示：不要迷戀容貌出眾者，修行後才知外表的前世因緣！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>地藏王菩薩開示：頭七超度的重要意義，這七天對亡者至關重要。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -5922,7 +5926,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>2025-06-22 16:59:14</t>
+          <t>2025-06-16 16:59:14</t>
         </is>
       </c>
     </row>
@@ -5934,7 +5938,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>文殊菩薩開示：修行人每天早上醒來，一定要先想這五件事！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>地藏王菩薩點化：想要來世有善報的人，今生要常做這五件事！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -5945,7 +5949,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>2025-07-21 04:59:14</t>
+          <t>2025-07-14 04:59:14</t>
         </is>
       </c>
     </row>
@@ -5957,7 +5961,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>文殊菩薩開示：在家居士最容易犯的三個錯誤，小心毀掉你的福報。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>地藏王菩薩：少跟孩子置氣，他們選擇你為父母，有這三種原因！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -5968,7 +5972,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>2025-06-22 22:59:14</t>
+          <t>2025-06-16 22:59:14</t>
         </is>
       </c>
     </row>
@@ -5980,7 +5984,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>文殊菩薩開示：錢財具有靈性，銘記4句真言能財富相隨！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>堅持素食的修行人，吃素背後到底是真修行，還是執念一場？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -5991,7 +5995,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>2025-06-23 04:59:14</t>
+          <t>2025-09-29 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6003,7 +6007,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>文殊菩薩點化：君子之交淡如水，佛門中的交友之道令人深思！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>外道沙門師傅詆毀佛法，眾比丘憤而議論，佛陀的教誨令所有人頓悟。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -6014,7 +6018,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>2025-06-23 10:59:14</t>
+          <t>2025-06-17 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6026,7 +6030,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>普賢菩薩十大行願，為何會獨缺一行，這個空白隱含什麽修行奧秘。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>大勢至菩薩開示：人在投胎前，為何會自己選擇父母，背後原因令人深思。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -6037,7 +6041,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>2025-06-23 16:59:14</t>
+          <t>2025-06-17 10:59:14</t>
         </is>
       </c>
     </row>
@@ -6049,7 +6053,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>普賢菩薩開示，一即一切，一切即一，其中蘊含佛法發人深省。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>大勢至菩薩開示：末法時代紛擾世界，保持內心平靜的終極奧秘！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -6058,7 +6062,11 @@
       <c r="D108" t="n">
         <v>1</v>
       </c>
-      <c r="E108" t="inlineStr"/>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>2025-06-17 16:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -6068,7 +6076,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>智光禪師臨終前點撥，福報只有一條路可獲得，那就是放棄福報！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>大勢至菩薩點化：當六根不凈時，這個修行秘訣讓你立刻心如止水。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -6079,7 +6087,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>2025-06-23 22:59:14</t>
+          <t>2025-06-17 22:59:14</t>
         </is>
       </c>
     </row>
@@ -6091,7 +6099,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>最强菩萨，地獄之主普渡眾生，20分鐘徹底了解地藏王菩薩。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>大梵天王問佛陀：何為空中妙有？佛陀回答揭示覺知奧秘。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -6102,7 +6110,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>2025-06-24 04:59:14</t>
+          <t>2025-06-18 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6114,7 +6122,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>最疼愛你的母親，竟是前世被你傷害過的人，佛陀開示因果輪回奧妙。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>大迦葉入定揭秘：原來十方佛土之外，眾生不過瞬息泡影！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -6125,7 +6133,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>2025-06-24 10:59:14</t>
+          <t>2025-09-30 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6137,7 +6145,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>末法時代修行人必看，踏入這五種學佛誤區，只會讓佛菩薩越來越遠。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>大迦葉問佛陀，為何修行人要斷除色欲？元神外泄導致修行受阻。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -6156,7 +6164,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>末法時代如何修行？釋迦牟尼開示阿難，這三種人最易圓滿！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>大迦葉問佛陀：為何亡者於人間徘徊七日，佛陀揭示陰陽兩界奧秘。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -6167,7 +6175,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>2025-06-24 16:59:14</t>
+          <t>2025-06-18 10:59:14</t>
         </is>
       </c>
     </row>
@@ -6179,7 +6187,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>末法時期如何修行？佛陀與藥師如來對話，揭示化解病苦的三大法門。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>大迦葉問釋迦牟尼，來世輪迴之說如何印證？佛陀的回答讓眾弟子沉默。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -6190,7 +6198,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>2025-06-24 22:59:14</t>
+          <t>2025-10-01 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6202,7 +6210,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>極樂世界唯一通行證，燃燈古佛揭示：沒有此秘訣，念佛萬遍也枉然！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>大迦葉問釋迦牟尼：如何“轉識成智”？佛陀開示：八識凈處五智自顯#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -6213,7 +6221,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>2025-07-22 04:59:14</t>
+          <t>2025-10-02 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6233,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>比丘問佛陀：色即是空，既然諸色皆空，為何修行之人要遠離女色。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>大迦葉問釋迦牟尼：成佛前為何要履行生子義務？真相讓所有人覺悟！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -6236,7 +6244,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>2025-06-25 04:59:14</t>
+          <t>2025-06-18 16:59:14</t>
         </is>
       </c>
     </row>
@@ -6248,7 +6256,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>比丘問釋迦牟尼，何為眾生平等四相皆空，佛陀開示人同狗並無分別。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>夫妻合葬輪迴後就能相見？地藏王菩薩說：來世能否重逢看這三件事！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -6259,7 +6267,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>2025-06-25 10:59:14</t>
+          <t>2025-07-15 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6271,7 +6279,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>比丘尼問釋迦牟尼：女人為何難成佛？佛陀開示讓眾人豁然開朗。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>女子跪問佛陀，為何不能散父親骨灰？佛陀揭示輪回奧秘。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -6282,7 +6290,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>2025-06-25 16:59:14</t>
+          <t>2025-06-18 22:59:14</t>
         </is>
       </c>
     </row>
@@ -6294,7 +6302,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>波斯匿王問佛陀：為何布施越多福報越少，一個故事點破布施因果奧妙。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>如何才能一念可成佛，佛陀揭示“心想事成”的奧秘，凡人如何修出神通？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -6305,7 +6313,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>2025-06-25 22:59:14</t>
+          <t>2025-10-03 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6317,7 +6325,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>波斯匿迦問佛陀，「我」究竟是什麽？，佛陀開示無我觀的奧秘。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>學佛之人切記，千萬別做這三件事，會耗光你的福報。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -6326,7 +6334,11 @@
       <c r="D120" t="n">
         <v>1</v>
       </c>
-      <c r="E120" t="inlineStr"/>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>2025-06-19 04:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -6336,7 +6348,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>涅槃寂靜，佛陀親授的終極解脫奧祕，一念之間超越生死。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>學佛人不可不知，佛前十種供品的寓意和果報，正確供養才能修行圓滿。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -6345,7 +6357,11 @@
       <c r="D121" t="n">
         <v>1</v>
       </c>
-      <c r="E121" t="inlineStr"/>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>2025-06-19 10:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -6355,7 +6371,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>為什麼好人沒好報？高僧秘密開示：福報被“偷走”的3個徵兆！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>家裡有“髒東西”怎麼辦？持念這一佛教咒語，驅邪避凶最為靈驗！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -6366,7 +6382,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>2025-06-26 04:59:14</t>
+          <t>2025-06-19 16:59:14</t>
         </is>
       </c>
     </row>
@@ -6378,7 +6394,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>為什麽「空」是佛教的核心智慧？揭秘「四大皆空」的真諦。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>富樓那問釋迦牟尼：您說無生無滅，那麽哪來的六道輪回呢？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -6389,7 +6405,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>2025-07-23 04:59:14</t>
+          <t>2025-06-19 22:59:14</t>
         </is>
       </c>
     </row>
@@ -6401,7 +6417,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>為什麽佛經讓人「讀不懂」？學會這7點就能輕松開啟智慧之門！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>已故親人會思念陽間人嗎？地藏王菩薩開示：時常思念但多數人不知！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -6412,7 +6428,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>2025-07-24 04:59:14</t>
+          <t>2025-07-16 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6424,7 +6440,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>為什麽佛說法四十九年，未曾說過一字？卻點亮無量眾生智慧，真相讓人驚嘆！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>帝釋天三問釋迦牟尼：「何為善」？佛陀的回答揭示人生大智慧。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -6435,7 +6451,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>2025-06-26 10:59:14</t>
+          <t>2025-06-20 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6463,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>為什麽佛陀說：持咒不如修心？一個漁夫的故事道破了修行的奥秘。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>帝釋天三問釋迦牟尼：輪回的盡頭是什麽？佛陀的開示令所有人頓悟！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -6458,7 +6474,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>2025-06-26 16:59:14</t>
+          <t>2025-06-20 10:59:14</t>
         </is>
       </c>
     </row>
@@ -6470,7 +6486,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>為什麽說「十小咒」擁有無量功德？短短幾句就能往生極樂，祛病消災福慧雙增#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>帝釋天問佛陀：何為菩提心？佛陀只用三個字，讓在場修行者瞬間開悟。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -6481,7 +6497,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>2025-06-26 22:59:14</t>
+          <t>2025-06-20 16:59:14</t>
         </is>
       </c>
     </row>
@@ -6493,7 +6509,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>為何佛陀涅槃後，大迦葉與阿難爆發激烈爭執？竟藏著佛教分裂真相。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>廣欽老和尚開示，如何做到一心不亂，領悟這三點當下即解脫！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -6504,7 +6520,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>2025-06-27 04:59:14</t>
+          <t>2025-06-20 22:59:14</t>
         </is>
       </c>
     </row>
@@ -6516,7 +6532,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>為何大德都說，2025年正月要誦讀金剛經？竟然蘊含著轉運玄機。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>彌勒佛問佛陀，何為究竟解脫，一句話讓眾人頓悟涅槃。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -6527,7 +6543,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>2025-06-27 10:59:14</t>
+          <t>2025-06-21 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6539,7 +6555,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>為何布施不宜張揚？觀世音菩薩開示：行善之時應當具足這三德！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>彌勒佛開示：人世間最大的布施，不是錢財而是這四個字！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -6550,7 +6566,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>2025-07-25 04:59:14</t>
+          <t>2025-07-17 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6578,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>為何高僧大德皆言，春節要讀地藏經？原來暗含這個修行機緣。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>彌勒菩薩問佛陀：未來的世界會怎樣？佛陀精準“預言”了人類的歸宿！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -6573,7 +6589,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>2025-07-26 04:59:14</t>
+          <t>2025-10-04 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6585,7 +6601,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>犯淫邪遭因果報應，高僧開示掌握此法，不僅可轉運還會發財！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>彌勒菩薩指引，轉世的真諦是什麼？超越生死才是究竟解脫！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -6596,7 +6612,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>2025-07-27 04:59:14</t>
+          <t>2025-06-21 10:59:14</t>
         </is>
       </c>
     </row>
@@ -6608,7 +6624,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>現今所說的四大皆空理念竟是錯誤的，這才是佛教「緣起論」的真正邏輯！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>心經中“究竟涅槃”的境界是什麼？大勢至菩薩的開示，讓眾人悟道修行真諦。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -6619,7 +6635,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>2025-06-27 16:59:14</t>
+          <t>2025-06-21 16:59:14</t>
         </is>
       </c>
     </row>
@@ -6631,7 +6647,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>目犍連問佛陀：親人真的會在六道重逢嗎？佛陀的開示讓眾人淚目！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>念《心經》前要先念開經偈嗎？文殊菩薩說順序錯了，念再多也沒用！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -6642,7 +6658,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>2025-06-27 22:59:14</t>
+          <t>2025-10-05 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6654,7 +6670,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>目犍連示現五神通，佛陀告誡弟子，修行為解脫而非神通。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>念佛不見佛現身，我們到底在求誰，禪師點破道理妙不可言！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -6665,7 +6681,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>2025-06-28 04:59:14</t>
+          <t>2025-06-21 22:59:14</t>
         </is>
       </c>
     </row>
@@ -6677,7 +6693,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>禪宗千年難題，執著與放下之間，如何找到菩提之路？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>念佛人的死後因果，觀世音菩薩揭秘：念佛次數決定往生品位！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -6688,7 +6704,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>2025-06-28 10:59:14</t>
+          <t>2025-07-18 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6700,7 +6716,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>禪宗藏著四句改命偈語，懂一句便可轉運，看看你能悟透幾句！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>念佛的真正目的！佛陀：不是“去”極樂，而是“發現”它！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -6711,7 +6727,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>2025-07-28 04:59:14</t>
+          <t>2025-10-06 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6723,7 +6739,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>禪定大師點撥：悟得這三個境界，可獲內心平靜通達涅槃境界！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>意淫比實淫更損元氣，未除此障修行難成就，學會此法可根除！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -6734,7 +6750,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>2025-07-29 04:59:14</t>
+          <t>2025-07-19 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6746,7 +6762,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>維摩詰假病示疾，揭露「在家成佛」的五個陷阱！你踩中幾條？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>成佛後還會輪迴嗎？這個終極問題的答案，揭示了佛性的永恆奧秘！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -6757,7 +6773,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>2025-06-28 16:59:14</t>
+          <t>2025-10-07 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6769,7 +6785,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>維摩詰問佛陀：在家與出家修行有何不同？佛陀一語道破精進要訣。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>探索密教深奧智慧！揭示寧瑪派傳世秘法與大圓滿修行的真實內涵！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -6780,7 +6796,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>2025-06-28 22:59:14</t>
+          <t>2025-06-22 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6808,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>維摩詰問佛陀：生死之間究竟相隔多遠？佛陀用一片落葉揭示輪回。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>揭開「阿彌陀佛」與「釋迦牟尼佛」的神秘關系，讓你徹底理解佛教宇宙的無盡智慧。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -6803,7 +6819,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>2025-06-29 04:59:14</t>
+          <t>2025-07-20 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6815,7 +6831,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>維摩詰居士開示：修行中的三種智慧，證悟三智方能照見本心！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>文殊菩薩問釋迦牟尼：何為無上正覺？佛陀的回答讓众人醍醐灌頂。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -6826,7 +6842,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>2025-07-30 04:59:14</t>
+          <t>2025-06-22 10:59:14</t>
         </is>
       </c>
     </row>
@@ -6838,7 +6854,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>維摩詰與佛陀的終極爭論：斷欲與親情如何兩全？佛陀回答顛覆認知！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>文殊菩薩問釋迦牟尼：智慧從何而來？佛陀微笑道出四字真言！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -6849,7 +6865,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>2025-07-31 04:59:14</t>
+          <t>2025-10-08 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6861,7 +6877,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>維摩詰開示弟子：做善事也會損耗福德，這四個標準才是行善關鍵。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>文殊菩薩開示：不要迷戀容貌出眾者，修行後才知外表的前世因緣！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -6872,7 +6888,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>2025-06-29 10:59:14</t>
+          <t>2025-06-22 16:59:14</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6900,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>老者問彌勒佛：酒肉穿腸過，佛祖心中留，這句話到底對不對？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>文殊菩薩開示：修行人每天早上醒來，一定要先想這五件事！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -6895,7 +6911,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>2025-08-01 04:59:14</t>
+          <t>2025-07-21 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6907,7 +6923,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>耆婆問釋迦牟尼：為何病人會痛苦？佛陀回答道出了生命真諦。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>文殊菩薩開示：在家居士最容易犯的三個錯誤，小心毀掉你的福報。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -6918,7 +6934,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>2025-06-29 16:59:14</t>
+          <t>2025-06-22 22:59:14</t>
         </is>
       </c>
     </row>
@@ -6930,7 +6946,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>舍利弗問釋迦牟尼：世尊您教導無住無執，為何又要世人皈依三寶。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>文殊菩薩開示：真正開悟的人具備，無中生有的能力和有中生無的智慧！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -6941,7 +6957,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>2025-06-29 22:59:14</t>
+          <t>2025-10-09 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6953,7 +6969,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>萬法歸宗，必有一得：三千年佛法智慧精華，藏在這四重心境之中！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>文殊菩薩開示：錢財具有靈性，銘記4句真言能財富相隨！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -6964,7 +6980,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>2025-08-02 04:59:14</t>
+          <t>2025-06-23 04:59:14</t>
         </is>
       </c>
     </row>
@@ -6976,16 +6992,20 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>虛空藏菩薩財富法，傳授五大富貴秘訣，第四訣改變命運軌跡。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>文殊菩薩點化：君子之交淡如水，佛門中的交友之道令人深思！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D149" t="n">
-        <v>0</v>
-      </c>
-      <c r="E149" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>2025-06-23 10:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -6995,7 +7015,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>西方極樂世界真的存在嗎？該如如何到達？原來也沒那麽難。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>普賢菩薩十大行願，為何會獨缺一行，這個空白隱含什麽修行奧秘。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -7004,7 +7024,11 @@
       <c r="D150" t="n">
         <v>1</v>
       </c>
-      <c r="E150" t="inlineStr"/>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>2025-06-23 16:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -7014,7 +7038,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>觀世音菩薩問佛陀：人死後真的會投胎嗎？佛陀的開示讓人徹悟。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>普賢菩薩問佛陀：如何才能生生世世修福報？佛陀的行願法門，讓你事半功倍！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -7025,7 +7049,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>2025-06-30 04:59:14</t>
+          <t>2025-10-10 04:59:14</t>
         </is>
       </c>
     </row>
@@ -7037,7 +7061,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>觀世音菩薩開示：老天要渡化你，會給你五種提醒，要留意！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>普賢菩薩開示，一即一切，一切即一，其中蘊含佛法發人深省。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -7046,11 +7070,7 @@
       <c r="D152" t="n">
         <v>1</v>
       </c>
-      <c r="E152" t="inlineStr">
-        <is>
-          <t>2025-06-30 10:59:14</t>
-        </is>
-      </c>
+      <c r="E152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -7060,7 +7080,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>觀音菩薩為什麽會由男變女？一個視頻講透觀世音的來歷和發展。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>智光禪師臨終前點撥，福報只有一條路可獲得，那就是放棄福報！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -7071,7 +7091,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>2025-08-03 04:59:14</t>
+          <t>2025-06-23 22:59:14</t>
         </is>
       </c>
     </row>
@@ -7083,7 +7103,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>觀音菩薩開示：供奉佛像時四個禁忌，很多人不知道一直在犯。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>最强菩萨，地獄之主普渡眾生，20分鐘徹底了解地藏王菩薩。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -7094,7 +7114,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>2025-06-30 16:59:14</t>
+          <t>2025-06-24 04:59:14</t>
         </is>
       </c>
     </row>
@@ -7106,7 +7126,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>觀音菩薩開示：真正有慈悲之人，不是天天拜佛，而是具有這三種品性。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>最疼愛你的母親，竟是前世被你傷害過的人，佛陀開示因果輪回奧妙。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -7115,7 +7135,11 @@
       <c r="D155" t="n">
         <v>1</v>
       </c>
-      <c r="E155" t="inlineStr"/>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>2025-06-24 10:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -7125,7 +7149,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>觀音菩薩點化善財：心中有佛也有魔，究竟如何才能超越二者？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>末法時代修行人必看，踏入這五種學佛誤區，只會讓佛菩薩越來越遠。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -7134,11 +7158,7 @@
       <c r="D156" t="n">
         <v>1</v>
       </c>
-      <c r="E156" t="inlineStr">
-        <is>
-          <t>2025-08-04 04:59:14</t>
-        </is>
-      </c>
+      <c r="E156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -7148,7 +7168,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>解讀《心經》，何爲“般若波羅蜜”，領悟佛法的終極智慧。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>末法時代如何修行？釋迦牟尼開示阿難，這三種人最易圓滿！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -7159,7 +7179,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>2025-06-30 22:59:14</t>
+          <t>2025-06-24 16:59:14</t>
         </is>
       </c>
     </row>
@@ -7171,7 +7191,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>言多語失造口業，觀音菩薩開示：修習這三種口德可避災禍！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>末法時期如何修行？佛陀與藥師如來對話，揭示化解病苦的三大法門。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -7182,7 +7202,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>2025-07-01 04:59:14</t>
+          <t>2025-06-24 22:59:14</t>
         </is>
       </c>
     </row>
@@ -7194,7 +7214,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>講透「五蘊皆空」真相，佛教智慧如何教你看透人生。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>極樂世界唯一通行證，燃燈古佛揭示：沒有此秘訣，念佛萬遍也枉然！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -7205,7 +7225,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>2025-08-05 04:59:14</t>
+          <t>2025-07-22 04:59:14</t>
         </is>
       </c>
     </row>
@@ -7217,7 +7237,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>超度亡者時，是念「地藏經」，還是念「往生咒」，高僧開示區別很大。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>比丘問佛陀：色即是空，既然諸色皆空，為何修行之人要遠離女色。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -7228,7 +7248,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>2025-07-01 10:59:14</t>
+          <t>2025-06-25 04:59:14</t>
         </is>
       </c>
     </row>
@@ -7240,7 +7260,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>迦旃延問釋迦牟尼：世尊您教導無相，為何又要世人供養佛像。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>比丘問釋迦牟尼，何為眾生平等四相皆空，佛陀開示人同狗並無分別。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -7251,7 +7271,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>2025-07-01 16:59:14</t>
+          <t>2025-06-25 10:59:14</t>
         </is>
       </c>
     </row>
@@ -7263,7 +7283,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>達摩祖師對慧可說：修行千萬別碰這四種“禪病”，否則終生困於幻境！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>比丘尼問釋迦牟尼：女人為何難成佛？佛陀開示讓眾人豁然開朗。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -7274,7 +7294,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>2025-08-06 04:59:14</t>
+          <t>2025-06-25 16:59:14</t>
         </is>
       </c>
     </row>
@@ -7286,7 +7306,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>達摩祖師點化弟子：參禪難在求玄妙，悟得此道方為妙法。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>波斯匿王問佛陀：為何布施越多福報越少，一個故事點破布施因果奧妙。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -7297,7 +7317,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>2025-07-01 22:59:14</t>
+          <t>2025-06-25 22:59:14</t>
         </is>
       </c>
     </row>
@@ -7309,7 +7329,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>釋迦牟尼佛為何斷言人生皆苦？十分鐘講透佛教四聖諦真相#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>波斯匿迦問佛陀，「我」究竟是什麽？，佛陀開示無我觀的奧秘。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -7318,11 +7338,7 @@
       <c r="D164" t="n">
         <v>1</v>
       </c>
-      <c r="E164" t="inlineStr">
-        <is>
-          <t>2025-07-02 04:59:14</t>
-        </is>
-      </c>
+      <c r="E164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -7332,7 +7348,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>釋迦牟尼：真正開悟的人都會具有這三種狀態。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>涅槃寂靜，佛陀親授的終極解脫奧祕，一念之間超越生死。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -7341,11 +7357,7 @@
       <c r="D165" t="n">
         <v>1</v>
       </c>
-      <c r="E165" t="inlineStr">
-        <is>
-          <t>2025-08-07 04:59:14</t>
-        </is>
-      </c>
+      <c r="E165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -7355,7 +7367,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>阿難問佛陀：人心如何才能不散亂？佛陀指出了日常生活中的修行法。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>為什麼好人沒好報？高僧秘密開示：福報被“偷走”的3個徵兆！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -7366,7 +7378,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>2025-08-08 04:59:14</t>
+          <t>2025-06-26 04:59:14</t>
         </is>
       </c>
     </row>
@@ -7378,7 +7390,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>阿難問佛陀：面對災禍，佛菩薩為何不普渡眾生，原來這兩種情況無法救度。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>為什麽「空」是佛教的核心智慧？揭秘「四大皆空」的真諦。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -7389,7 +7401,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>2025-08-09 04:59:14</t>
+          <t>2025-07-23 04:59:14</t>
         </is>
       </c>
     </row>
@@ -7401,7 +7413,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>阿難問釋迦牟尼佛：涅槃是新生還是他生？佛陀回答讓眾生頓悟！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>為什麽佛經讓人「讀不懂」？學會這7點就能輕松開啟智慧之門！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -7412,7 +7424,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>2025-08-10 04:59:14</t>
+          <t>2025-07-24 04:59:14</t>
         </is>
       </c>
     </row>
@@ -7424,7 +7436,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>阿難問釋迦牟尼，如何區分真假開悟，佛陀用四句話讓眾人徹悟！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>為什麽佛說法四十九年，未曾說過一字？卻點亮無量眾生智慧，真相讓人驚嘆！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -7433,7 +7445,11 @@
       <c r="D169" t="n">
         <v>1</v>
       </c>
-      <c r="E169" t="inlineStr"/>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>2025-06-26 10:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -7443,7 +7459,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>阿難問釋迦牟尼：世尊為何不開創凈土？佛陀的回答讓人頓悟。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>為什麽佛陀說：持咒不如修心？一個漁夫的故事道破了修行的奥秘。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -7454,7 +7470,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>2025-08-11 04:59:14</t>
+          <t>2025-06-26 16:59:14</t>
         </is>
       </c>
     </row>
@@ -7466,7 +7482,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>阿難問釋迦牟尼：人為何會有生死？佛陀回答道出生死真相。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>為什麽說「十小咒」擁有無量功德？短短幾句就能往生極樂，祛病消災福慧雙增#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -7477,7 +7493,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>2025-08-12 04:59:14</t>
+          <t>2025-06-26 22:59:14</t>
         </is>
       </c>
     </row>
@@ -7489,7 +7505,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>阿難問釋迦牟尼：您涅槃之後還會輪回嗎？佛陀的回答令眾生頓悟。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>為何佛陀涅槃後，大迦葉與阿難爆發激烈爭執？竟藏著佛教分裂真相。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -7500,7 +7516,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>2025-08-13 04:59:14</t>
+          <t>2025-06-27 04:59:14</t>
         </is>
       </c>
     </row>
@@ -7512,7 +7528,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>阿難問釋迦牟尼：為何修行人也做春夢？佛陀揭示三個不為人知的原因！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>為何大德都說，2025年正月要誦讀金剛經？竟然蘊含著轉運玄機。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -7523,7 +7539,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>2025-08-14 04:59:14</t>
+          <t>2025-06-27 10:59:14</t>
         </is>
       </c>
     </row>
@@ -7535,7 +7551,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>阿難問釋迦牟尼：為何修行越深心魔越強？佛陀指出了關鍵盲點！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>為何布施不宜張揚？觀世音菩薩開示：行善之時應當具足這三德！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -7546,7 +7562,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>2025-08-15 04:59:14</t>
+          <t>2025-07-25 04:59:14</t>
         </is>
       </c>
     </row>
@@ -7558,7 +7574,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>阿難問：世尊教導不執著，為何對佛法如此珍重？佛陀回答令人深思。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>為何念佛時會突然流淚？阿彌陀佛親示：往生前的五種殊勝徵兆#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -7569,7 +7585,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>2025-08-16 04:59:14</t>
+          <t>2025-10-11 04:59:14</t>
         </is>
       </c>
     </row>
@@ -7581,7 +7597,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>阿難尊者親歷，觀世音菩薩顯靈傳授，讓祈求必成的三個發願法則！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>為何高僧大德皆言，春節要讀地藏經？原來暗含這個修行機緣。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -7590,7 +7606,11 @@
       <c r="D176" t="n">
         <v>1</v>
       </c>
-      <c r="E176" t="inlineStr"/>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>2025-07-26 04:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -7600,7 +7620,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>阿難開示比丘，心淫比身淫更傷修行，領悟此法可助斷欲修身。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>無量壽佛講經說法：極樂世界不是玄幻，做到這幾點必定往生!#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -7611,7 +7631,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>2025-08-17 04:59:14</t>
+          <t>2025-10-12 04:59:14</t>
         </is>
       </c>
     </row>
@@ -7623,7 +7643,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>隨喜加入，同修善法，南無阿彌陀佛！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>犯淫邪遭因果報應，高僧開示掌握此法，不僅可轉運還會發財！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -7634,7 +7654,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>2025-08-18 04:59:14</t>
+          <t>2025-07-27 04:59:14</t>
         </is>
       </c>
     </row>
@@ -7646,7 +7666,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>須菩提問佛陀，什麽是「無生法忍」，文殊菩薩道破修行終極奧義。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>現今所說的四大皆空理念竟是錯誤的，這才是佛教「緣起論」的真正邏輯！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -7655,7 +7675,11 @@
       <c r="D179" t="n">
         <v>1</v>
       </c>
-      <c r="E179" t="inlineStr"/>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>2025-06-27 16:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -7665,7 +7689,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>須菩提問佛陀：世間苦難何時了？佛陀妙語開示眾人醒悟！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>目犍連問佛陀：親人真的會在六道重逢嗎？佛陀的開示讓眾人淚目！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -7674,7 +7698,11 @@
       <c r="D180" t="n">
         <v>1</v>
       </c>
-      <c r="E180" t="inlineStr"/>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>2025-06-27 22:59:14</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -7684,7 +7712,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>須達多問佛陀：為何好人早逝，惡人長壽，一個故事揭開三世因果真相。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>目犍連問釋迦牟尼：地獄景象究竟是實有還是心造？佛陀的回答令眾生頓悟!#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -7695,7 +7723,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>2025-08-19 04:59:14</t>
+          <t>2025-10-13 04:59:14</t>
         </is>
       </c>
     </row>
@@ -7707,7 +7735,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>須達多問釋迦牟尼：佛陀您教導布施，為何還要弟子日日托缽。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>目犍連示現五神通，佛陀告誡弟子，修行為解脫而非神通。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -7718,7 +7746,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>2025-08-20 04:59:14</t>
+          <t>2025-06-28 04:59:14</t>
         </is>
       </c>
     </row>
@@ -7730,7 +7758,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>颠覆你对佛法的认知！99%的人都误解的修行真相，佛教真正的秘密首次揭露！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>禪宗千年難題，執著與放下之間，如何找到菩提之路？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -7741,7 +7769,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>2025-08-21 04:59:14</t>
+          <t>2025-06-28 10:59:14</t>
         </is>
       </c>
     </row>
@@ -7753,7 +7781,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>體內住著兩個“自己”？佛陀：識得“元神”，方能跳出輪迴！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>禪宗藏著四句改命偈語，懂一句便可轉運，看看你能悟透幾句！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -7764,7 +7792,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>2025-08-22 04:59:14</t>
+          <t>2025-07-28 04:59:14</t>
         </is>
       </c>
     </row>
@@ -7776,7 +7804,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>高僧警示修行人，修得越精業力反噬越狠，很多人敗在證悟前一刻！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>禪定大師點撥：悟得這三個境界，可獲內心平靜通達涅槃境界！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -7787,7 +7815,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>2025-08-23 04:59:14</t>
+          <t>2025-07-29 04:59:14</t>
         </is>
       </c>
     </row>
@@ -7799,7 +7827,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>鬼怕哪種人？佛說：有3種人，連鬼也不敢靠近他！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>維摩詰假病示疾，揭露「在家成佛」的五個陷阱！你踩中幾條？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -7810,7 +7838,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>2025-08-24 04:59:14</t>
+          <t>2025-06-28 16:59:14</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7850,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>魔王波旬問佛陀：殺業深重者能否成佛？佛陀用一句話點化極惡眾生！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>維摩詰問佛陀：在家與出家修行有何不同？佛陀一語道破精進要訣。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -7833,7 +7861,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>2025-08-25 04:59:14</t>
+          <t>2025-06-28 22:59:14</t>
         </is>
       </c>
     </row>
@@ -7845,7 +7873,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>龍樹菩薩與外道終極辯論：空性與實相如何兩全？答案直指萬法根源！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+          <t>維摩詰問佛陀：生死之間究竟相隔多遠？佛陀用一片落葉揭示輪回。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -7856,7 +7884,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>2025-08-26 04:59:14</t>
+          <t>2025-06-29 04:59:14</t>
         </is>
       </c>
     </row>
@@ -7868,16 +7896,1502 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
+          <t>維摩詰居士開示：修行中的三種智慧，證悟三智方能照見本心！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>1</v>
+      </c>
+      <c r="D189" t="n">
+        <v>1</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>2025-07-30 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>維摩詰與佛陀的終極爭論：斷欲與親情如何兩全？佛陀回答顛覆認知！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>1</v>
+      </c>
+      <c r="D190" t="n">
+        <v>1</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>2025-07-31 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>維摩詰開示弟子：做善事也會損耗福德，這四個標準才是行善關鍵。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>1</v>
+      </c>
+      <c r="D191" t="n">
+        <v>1</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>2025-06-29 10:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>老者問彌勒佛：酒肉穿腸過，佛祖心中留，這句話到底對不對？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>1</v>
+      </c>
+      <c r="D192" t="n">
+        <v>1</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>2025-08-01 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>耆婆問釋迦牟尼：為何病人會痛苦？佛陀回答道出了生命真諦。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>1</v>
+      </c>
+      <c r="D193" t="n">
+        <v>1</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>2025-06-29 16:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>舍利弗問釋迦牟尼，何為“真正的智慧”，佛陀開示智者的六個維度#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>1</v>
+      </c>
+      <c r="D194" t="n">
+        <v>1</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>2025-10-14 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>舍利弗問釋迦牟尼：世尊您教導無住無執，為何又要世人皈依三寶。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>1</v>
+      </c>
+      <c r="D195" t="n">
+        <v>1</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>2025-06-29 22:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>舍利弗問釋迦牟尼：臨終時是苦是樂？佛陀用八個字讓眾生頓悟!#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>1</v>
+      </c>
+      <c r="D196" t="n">
+        <v>1</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>2025-10-15 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>舍利弗問釋迦牟尼：過去諸佛涅槃後，去往了何處？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>1</v>
+      </c>
+      <c r="D197" t="n">
+        <v>1</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>2025-10-16 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>萬法歸宗，必有一得：三千年佛法智慧精華，藏在這四重心境之中！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>1</v>
+      </c>
+      <c r="D198" t="n">
+        <v>1</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>2025-08-02 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>虛空藏菩薩財富法，傳授五大富貴秘訣，第四訣改變命運軌跡。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>0</v>
+      </c>
+      <c r="D199" t="n">
+        <v>0</v>
+      </c>
+      <c r="E199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>西方極樂世界會消失嗎？佛陀揭示宇宙真相，顛覆你對極樂凈土的認知。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>1</v>
+      </c>
+      <c r="D200" t="n">
+        <v>1</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>2025-10-17 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>西方極樂世界為何分三品九等？龍樹菩薩示現揭秘：原來暗藏修行階梯等級!#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>1</v>
+      </c>
+      <c r="D201" t="n">
+        <v>1</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>2025-10-18 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>西方極樂世界真的存在嗎？玄奘法師臨終前揭秘，真相顛覆世人認知!#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
+        <v>1</v>
+      </c>
+      <c r="D202" t="n">
+        <v>1</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>2025-10-19 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>西方極樂世界真的存在嗎？該如如何到達？原來也沒那麽難。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>1</v>
+      </c>
+      <c r="D203" t="n">
+        <v>1</v>
+      </c>
+      <c r="E203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>觀世音菩薩問佛陀：人死後真的會投胎嗎？佛陀的開示讓人徹悟。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>1</v>
+      </c>
+      <c r="D204" t="n">
+        <v>1</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>2025-06-30 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>觀世音菩薩開示：老天要渡化你，會給你五種提醒，要留意！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>1</v>
+      </c>
+      <c r="D205" t="n">
+        <v>1</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>2025-06-30 10:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>觀世音菩薩顯靈開示：真學佛人不止於吃齋念佛，而在參透這五個修行關鍵!#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C206" t="n">
+        <v>1</v>
+      </c>
+      <c r="D206" t="n">
+        <v>1</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>2025-10-20 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>觀音菩薩問釋迦牟尼：為何世人常陷苦海？佛陀的答案解救了億萬眾生#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>1</v>
+      </c>
+      <c r="D207" t="n">
+        <v>1</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>2025-10-21 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>觀音菩薩為什麽會由男變女？一個視頻講透觀世音的來歷和發展。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>1</v>
+      </c>
+      <c r="D208" t="n">
+        <v>1</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>2025-08-03 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>觀音菩薩開示：供奉佛像時四個禁忌，很多人不知道一直在犯。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>1</v>
+      </c>
+      <c r="D209" t="n">
+        <v>1</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>2025-06-30 16:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>觀音菩薩開示：真正有慈悲之人，不是天天拜佛，而是具有這三種品性。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>1</v>
+      </c>
+      <c r="D210" t="n">
+        <v>1</v>
+      </c>
+      <c r="E210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>觀音菩薩點化善財：心中有佛也有魔，究竟如何才能超越二者？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>1</v>
+      </c>
+      <c r="D211" t="n">
+        <v>1</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>2025-08-04 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>解讀《心經》，何爲“般若波羅蜜”，領悟佛法的終極智慧。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>1</v>
+      </c>
+      <c r="D212" t="n">
+        <v>1</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>2025-06-30 22:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>言多語失造口業，觀音菩薩開示：修習這三種口德可避災禍！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>1</v>
+      </c>
+      <c r="D213" t="n">
+        <v>1</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>2025-07-01 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>講透「五蘊皆空」真相，佛教智慧如何教你看透人生。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>1</v>
+      </c>
+      <c r="D214" t="n">
+        <v>1</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>2025-08-05 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>超度亡者時，是念「地藏經」，還是念「往生咒」，高僧開示區別很大。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C215" t="n">
+        <v>1</v>
+      </c>
+      <c r="D215" t="n">
+        <v>1</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>2025-07-01 10:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>迦旃延問釋迦牟尼：世尊您教導無相，為何又要世人供養佛像。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C216" t="n">
+        <v>1</v>
+      </c>
+      <c r="D216" t="n">
+        <v>1</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>2025-07-01 16:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>迦葉問釋迦牟尼：您如何確定自己已成佛？佛陀回答讓人大徹大悟!#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C217" t="n">
+        <v>1</v>
+      </c>
+      <c r="D217" t="n">
+        <v>1</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>2025-10-22 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>達摩祖師對慧可說：修行千萬別碰這四種“禪病”，否則終生困於幻境！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C218" t="n">
+        <v>1</v>
+      </c>
+      <c r="D218" t="n">
+        <v>1</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>2025-08-06 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>達摩祖師點化弟子：參禪難在求玄妙，悟得此道方為妙法。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C219" t="n">
+        <v>1</v>
+      </c>
+      <c r="D219" t="n">
+        <v>1</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>2025-07-01 22:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>釋迦牟尼佛為何斷言人生皆苦？十分鐘講透佛教四聖諦真相#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C220" t="n">
+        <v>1</v>
+      </c>
+      <c r="D220" t="n">
+        <v>1</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>2025-07-02 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>釋迦牟尼佛講劫數：為什麼說時間是幻象？劫數背後隱藏什麼？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C221" t="n">
+        <v>1</v>
+      </c>
+      <c r="D221" t="n">
+        <v>1</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>2025-10-23 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>釋迦牟尼佛講輪迴：為什麼說死亡只是幻覺？六道背後隱藏什麼秘密？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C222" t="n">
+        <v>1</v>
+      </c>
+      <c r="D222" t="n">
+        <v>1</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>2025-10-24 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>釋迦牟尼佛預言：末法時代能往生凈土的人，都具備這三種特質#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C223" t="n">
+        <v>1</v>
+      </c>
+      <c r="D223" t="n">
+        <v>0</v>
+      </c>
+      <c r="E223" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>釋迦牟尼臨終開示：末法時代將現幾種人，比魔王波旬可怕千百倍#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C224" t="n">
+        <v>1</v>
+      </c>
+      <c r="D224" t="n">
+        <v>1</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>2025-10-25 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>釋迦牟尼證悟後說出：輪迴最可怕的不是受苦，而是不知道自己在輪迴中#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C225" t="n">
+        <v>1</v>
+      </c>
+      <c r="D225" t="n">
+        <v>1</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>2025-10-26 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>釋迦牟尼：真正開悟的人都會具有這三種狀態。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C226" t="n">
+        <v>1</v>
+      </c>
+      <c r="D226" t="n">
+        <v>1</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>2025-08-07 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>阿彌陀佛垂訓：命終之時持誦這四字，可往生極樂永脫六道輪迴#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C227" t="n">
+        <v>1</v>
+      </c>
+      <c r="D227" t="n">
+        <v>1</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>2025-10-27 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>阿難問佛陀：人心如何才能不散亂？佛陀指出了日常生活中的修行法。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C228" t="n">
+        <v>1</v>
+      </c>
+      <c r="D228" t="n">
+        <v>1</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>2025-08-08 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>阿難問佛陀：面對災禍，佛菩薩為何不普渡眾生，原來這兩種情況無法救度。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C229" t="n">
+        <v>1</v>
+      </c>
+      <c r="D229" t="n">
+        <v>1</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>2025-08-09 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>阿難問觀音菩薩：情慾既是輪迴之因，那夫妻恩愛也是罪業嗎？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C230" t="n">
+        <v>1</v>
+      </c>
+      <c r="D230" t="n">
+        <v>1</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>2025-10-28 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>阿難問釋迦牟尼佛：涅槃是新生還是他生？佛陀回答讓眾生頓悟！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C231" t="n">
+        <v>1</v>
+      </c>
+      <c r="D231" t="n">
+        <v>1</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>2025-08-10 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>阿難問釋迦牟尼，“生死事大，無常迅速”何解？佛陀開示讓眾弟子覺悟#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C232" t="n">
+        <v>1</v>
+      </c>
+      <c r="D232" t="n">
+        <v>1</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>2025-10-29 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>阿難問釋迦牟尼，如何區分真假開悟，佛陀用四句話讓眾人徹悟！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C233" t="n">
+        <v>1</v>
+      </c>
+      <c r="D233" t="n">
+        <v>1</v>
+      </c>
+      <c r="E233" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>阿難問釋迦牟尼：世尊為何不開創凈土？佛陀的回答讓人頓悟。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C234" t="n">
+        <v>1</v>
+      </c>
+      <c r="D234" t="n">
+        <v>1</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>2025-08-11 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>阿難問釋迦牟尼：人為何會有生死？佛陀回答道出生死真相。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C235" t="n">
+        <v>1</v>
+      </c>
+      <c r="D235" t="n">
+        <v>1</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>2025-08-12 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>阿難問釋迦牟尼：佛法無邊，是否有您也無法闡釋的真理？佛陀的回答打破思維陷阱#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C236" t="n">
+        <v>1</v>
+      </c>
+      <c r="D236" t="n">
+        <v>1</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>2025-10-30 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>阿難問釋迦牟尼：您涅槃之後還會輪回嗎？佛陀的回答令眾生頓悟。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>1</v>
+      </c>
+      <c r="D237" t="n">
+        <v>1</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>2025-08-13 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>阿難問釋迦牟尼：為何修行人也做春夢？佛陀揭示三個不為人知的原因！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C238" t="n">
+        <v>1</v>
+      </c>
+      <c r="D238" t="n">
+        <v>1</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>2025-08-14 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>阿難問釋迦牟尼：為何修行越深心魔越強？佛陀指出了關鍵盲點！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C239" t="n">
+        <v>1</v>
+      </c>
+      <c r="D239" t="n">
+        <v>1</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>2025-08-15 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>阿難問：世尊教導不執著，為何對佛法如此珍重？佛陀回答令人深思。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>1</v>
+      </c>
+      <c r="D240" t="n">
+        <v>1</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>2025-08-16 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>阿難尊者親歷，觀世音菩薩顯靈傳授，讓祈求必成的三個發願法則！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C241" t="n">
+        <v>1</v>
+      </c>
+      <c r="D241" t="n">
+        <v>1</v>
+      </c>
+      <c r="E241" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>阿難開示比丘，心淫比身淫更傷修行，領悟此法可助斷欲修身。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C242" t="n">
+        <v>1</v>
+      </c>
+      <c r="D242" t="n">
+        <v>1</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>2025-08-17 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>隨喜加入，同修善法，南無阿彌陀佛！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C243" t="n">
+        <v>1</v>
+      </c>
+      <c r="D243" t="n">
+        <v>1</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>2025-08-18 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>須菩提問佛陀，什麽是「無生法忍」，文殊菩薩道破修行終極奧義。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C244" t="n">
+        <v>1</v>
+      </c>
+      <c r="D244" t="n">
+        <v>1</v>
+      </c>
+      <c r="E244" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>須菩提問佛陀：世間苦難何時了？佛陀妙語開示眾人醒悟！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C245" t="n">
+        <v>1</v>
+      </c>
+      <c r="D245" t="n">
+        <v>1</v>
+      </c>
+      <c r="E245" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>須菩提問佛陀：既然眾生都在輪迴，那最初的眾生是從何而來？#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C246" t="n">
+        <v>1</v>
+      </c>
+      <c r="D246" t="n">
+        <v>1</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>2025-10-31 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>須達多問佛陀：為何好人早逝，惡人長壽，一個故事揭開三世因果真相。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C247" t="n">
+        <v>1</v>
+      </c>
+      <c r="D247" t="n">
+        <v>1</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>2025-08-19 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>須達多問釋迦牟尼：佛陀您教導布施，為何還要弟子日日托缽。#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C248" t="n">
+        <v>1</v>
+      </c>
+      <c r="D248" t="n">
+        <v>1</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>2025-08-20 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>颠覆你对佛法的认知！99%的人都误解的修行真相，佛教真正的秘密首次揭露！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C249" t="n">
+        <v>1</v>
+      </c>
+      <c r="D249" t="n">
+        <v>1</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>2025-08-21 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>體內住著兩個“自己”？佛陀：識得“元神”，方能跳出輪迴！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C250" t="n">
+        <v>1</v>
+      </c>
+      <c r="D250" t="n">
+        <v>1</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>2025-08-22 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>高僧警示修行人，修得越精業力反噬越狠，很多人敗在證悟前一刻！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C251" t="n">
+        <v>1</v>
+      </c>
+      <c r="D251" t="n">
+        <v>1</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>2025-08-23 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>鬼怕哪種人？佛說：有3種人，連鬼也不敢靠近他！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C252" t="n">
+        <v>1</v>
+      </c>
+      <c r="D252" t="n">
+        <v>1</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>2025-08-24 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>魔王波旬問佛陀：殺業深重者能否成佛？佛陀用一句話點化極惡眾生！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C253" t="n">
+        <v>1</v>
+      </c>
+      <c r="D253" t="n">
+        <v>1</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>2025-08-25 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>龍樹菩薩與外道終極辯論：空性與實相如何兩全？答案直指萬法根源！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
+        </is>
+      </c>
+      <c r="C254" t="n">
+        <v>1</v>
+      </c>
+      <c r="D254" t="n">
+        <v>1</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>2025-08-26 04:59:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>佛道禪緣</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
           <t>龍樹菩薩開示：見性成佛的三重境界，開悟得解脫迷惑墮輪迴！#佛教 #佛家 #佛法 #佛學知識 #佛學智慧 #修心修行 #佛教文化 #禪悟人生 #傳統文化.mp4</t>
         </is>
       </c>
-      <c r="C189" t="n">
-        <v>1</v>
-      </c>
-      <c r="D189" t="n">
-        <v>1</v>
-      </c>
-      <c r="E189" t="inlineStr">
+      <c r="C255" t="n">
+        <v>1</v>
+      </c>
+      <c r="D255" t="n">
+        <v>1</v>
+      </c>
+      <c r="E255" t="inlineStr">
         <is>
           <t>2025-08-27 04:59:14</t>
         </is>

</xml_diff>